<commit_message>
Expand Ichalkaranji directory with 36 sourced business contacts
</commit_message>
<xml_diff>
--- a/services.xlsx
+++ b/services.xlsx
@@ -491,7 +491,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N67"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -1465,9 +1465,1179 @@
         <v>No</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="1" t="str">
+        <v>Hallmark Furniture</v>
+      </c>
+      <c r="B32" s="1" t="str">
+        <v>Furniture &amp; Installation</v>
+      </c>
+      <c r="C32" s="1" t="str">
+        <v>Home Interiors</v>
+      </c>
+      <c r="F32" s="1" t="str">
+        <v>+919337939393</v>
+      </c>
+      <c r="H32" s="1" t="str">
+        <v>Station Road, Ichalkaranji</v>
+      </c>
+      <c r="I32" s="1" t="str">
+        <v>Furniture sales, made-to-size furniture enquiries, delivery and installation</v>
+      </c>
+      <c r="K32" s="1" t="str">
+        <v>https://hallmarkfurniture.in/contact/</v>
+      </c>
+      <c r="L32" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M32" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N32" s="1" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="str">
+        <v>Jannat Interior</v>
+      </c>
+      <c r="B33" s="1" t="str">
+        <v>Wall Panels &amp; Interiors</v>
+      </c>
+      <c r="C33" s="1" t="str">
+        <v>Home Interiors</v>
+      </c>
+      <c r="F33" s="1" t="str">
+        <v>+919699575774</v>
+      </c>
+      <c r="H33" s="1" t="str">
+        <v>Ichalkaranji; also serves Kolhapur and Sangli</v>
+      </c>
+      <c r="I33" s="1" t="str">
+        <v>WPC and PVC wall-panel installation, false ceilings, TV units and home or office interiors</v>
+      </c>
+      <c r="J33" s="1" t="str">
+        <v>wall decoration, wall panels, ceiling work, भिंतीचे पॅनेल, इंटेरियर</v>
+      </c>
+      <c r="K33" s="1" t="str">
+        <v>https://jannatinterior.in/locations/ichalkaranji/</v>
+      </c>
+      <c r="L33" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M33" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N33" s="1" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="str">
+        <v>Gurukrupa Electronics &amp; Electricals</v>
+      </c>
+      <c r="B34" s="1" t="str">
+        <v>Appliance Sales &amp; Support</v>
+      </c>
+      <c r="C34" s="1" t="str">
+        <v>Appliances &amp; Electronics</v>
+      </c>
+      <c r="F34" s="1" t="str">
+        <v>+919921243457</v>
+      </c>
+      <c r="H34" s="1" t="str">
+        <v>Ichalkaranji stores</v>
+      </c>
+      <c r="I34" s="1" t="str">
+        <v>Enquiries and customer support for TVs, washing machines, refrigerators, ACs, laptops and mobiles</v>
+      </c>
+      <c r="K34" s="1" t="str">
+        <v>https://gurukrupaelectronics.com/</v>
+      </c>
+      <c r="L34" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M34" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N34" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="str">
+        <v>Vastu Construction</v>
+      </c>
+      <c r="B35" s="1" t="str">
+        <v>Construction &amp; Interior Design</v>
+      </c>
+      <c r="C35" s="1" t="str">
+        <v>Home Interiors</v>
+      </c>
+      <c r="F35" s="1" t="str">
+        <v>+919604459628</v>
+      </c>
+      <c r="H35" s="1" t="str">
+        <v>Kamble Building, Satpute Galli, near Ram Mandir, Ichalkaranji</v>
+      </c>
+      <c r="I35" s="1" t="str">
+        <v>Building planning, construction, interior and exterior design, and 3D design enquiries</v>
+      </c>
+      <c r="K35" s="1" t="str">
+        <v>https://www.vastu-constructions.com/index.html</v>
+      </c>
+      <c r="L35" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M35" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N35" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="str">
+        <v>OM Enterprises</v>
+      </c>
+      <c r="B36" s="1" t="str">
+        <v>Appliance Store</v>
+      </c>
+      <c r="C36" s="1" t="str">
+        <v>Appliances &amp; Electronics</v>
+      </c>
+      <c r="F36" s="1" t="str">
+        <v>+919762717096</v>
+      </c>
+      <c r="H36" s="1" t="str">
+        <v>Shahunagar Chandur, Line No. 4, Ichalkaranji area</v>
+      </c>
+      <c r="I36" s="1" t="str">
+        <v>Sales enquiries for refrigerators, TVs, washing machines, ACs, RO purifiers and printers</v>
+      </c>
+      <c r="K36" s="1" t="str">
+        <v>https://om-enterprises-in.ueniweb.com/</v>
+      </c>
+      <c r="L36" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M36" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N36" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="str">
+        <v>RK Water Solutions</v>
+      </c>
+      <c r="B37" s="1" t="str">
+        <v>Water Purifier Service</v>
+      </c>
+      <c r="C37" s="1" t="str">
+        <v>Repairs &amp; Maintenance</v>
+      </c>
+      <c r="F37" s="1" t="str">
+        <v>+917776932211</v>
+      </c>
+      <c r="H37" s="1" t="str">
+        <v>Panchganga Sugar Factory Road, opposite Panchratn Bhavan, Industrial Estate, Ichalkaranji</v>
+      </c>
+      <c r="I37" s="1" t="str">
+        <v>Domestic, commercial and industrial RO systems; purifier servicing, filter replacement and AMC enquiries</v>
+      </c>
+      <c r="J37" s="1" t="str">
+        <v>RO repair, water filter, purifier maintenance, पाणी फिल्टर, वॉटर प्युरिफायर</v>
+      </c>
+      <c r="K37" s="1" t="str">
+        <v>https://rkwatersolutions.in/</v>
+      </c>
+      <c r="L37" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M37" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N37" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="str">
+        <v>Jakbrillo Innovations</v>
+      </c>
+      <c r="B38" s="1" t="str">
+        <v>Laser Cutting &amp; Engraving</v>
+      </c>
+      <c r="C38" s="1" t="str">
+        <v>Business &amp; Technical Services</v>
+      </c>
+      <c r="F38" s="1" t="str">
+        <v>+912302431550</v>
+      </c>
+      <c r="H38" s="1" t="str">
+        <v>8, Rajarshi Shahu Market, Janta Chowk, Ichalkaranji</v>
+      </c>
+      <c r="I38" s="1" t="str">
+        <v>Laser cutting and engraving enquiries for textiles, curtains, acrylic, wood, paper and decorative work</v>
+      </c>
+      <c r="K38" s="1" t="str">
+        <v>https://jakbrillo.com/printmaterialprocessed.php</v>
+      </c>
+      <c r="L38" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M38" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N38" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="str">
+        <v>S.P. Engineers &amp; Suppliers</v>
+      </c>
+      <c r="B39" s="1" t="str">
+        <v>Electrical Contractor</v>
+      </c>
+      <c r="C39" s="1" t="str">
+        <v>Business &amp; Technical Services</v>
+      </c>
+      <c r="F39" s="1" t="str">
+        <v>+918483001718</v>
+      </c>
+      <c r="H39" s="1" t="str">
+        <v>12/581, near Dr. Sakharpe Hospital Chowk, Ichalkaranji</v>
+      </c>
+      <c r="I39" s="1" t="str">
+        <v>Industrial and commercial electrical design, installation, panels and commissioning</v>
+      </c>
+      <c r="K39" s="1" t="str">
+        <v>https://www.spevolution.com/</v>
+      </c>
+      <c r="L39" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M39" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N39" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="str">
+        <v>Goldenray Future Energy</v>
+      </c>
+      <c r="B40" s="1" t="str">
+        <v>Solar Projects</v>
+      </c>
+      <c r="C40" s="1" t="str">
+        <v>Solar &amp; Energy</v>
+      </c>
+      <c r="F40" s="1" t="str">
+        <v>+919049041500</v>
+      </c>
+      <c r="H40" s="1" t="str">
+        <v>Ichalkaranji office: Pritisangam Building, Saraswati Market area, Khanjire Mala</v>
+      </c>
+      <c r="I40" s="1" t="str">
+        <v>Commercial and industrial solar project enquiries, EPC and turnkey solar installations</v>
+      </c>
+      <c r="K40" s="1" t="str">
+        <v>https://www.goldenray.in/contact-us.php</v>
+      </c>
+      <c r="L40" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M40" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N40" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="str">
+        <v>Life Solar</v>
+      </c>
+      <c r="B41" s="1" t="str">
+        <v>Solar Installation &amp; Maintenance</v>
+      </c>
+      <c r="C41" s="1" t="str">
+        <v>Solar &amp; Energy</v>
+      </c>
+      <c r="F41" s="1" t="str">
+        <v>+918668824098</v>
+      </c>
+      <c r="H41" s="1" t="str">
+        <v>Saranagar, Rui-Ichalkaranji, Kolhapur district</v>
+      </c>
+      <c r="I41" s="1" t="str">
+        <v>Industrial, commercial and ground-mounted solar installation, engineering and maintenance enquiries</v>
+      </c>
+      <c r="K41" s="1" t="str">
+        <v>https://lifesolar.in/contact/</v>
+      </c>
+      <c r="L41" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M41" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N41" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="str">
+        <v>Indumati Solutions — Ichalkaranji</v>
+      </c>
+      <c r="B42" s="1" t="str">
+        <v>Facility Maintenance</v>
+      </c>
+      <c r="C42" s="1" t="str">
+        <v>Building Services</v>
+      </c>
+      <c r="F42" s="1" t="str">
+        <v>+919158887178</v>
+      </c>
+      <c r="H42" s="1" t="str">
+        <v>Pratik Plaza, opposite Hotel Upvan, Kolhapur Road, Ichalkaranji</v>
+      </c>
+      <c r="I42" s="1" t="str">
+        <v>Facility services, pest control, facade cleaning, gardening and landscaping enquiries</v>
+      </c>
+      <c r="K42" s="1" t="str">
+        <v>https://indumati.com/facility-mangement.html</v>
+      </c>
+      <c r="L42" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M42" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N42" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="str">
+        <v>Manisha Infotech</v>
+      </c>
+      <c r="B43" s="1" t="str">
+        <v>Computer &amp; CCTV Repair</v>
+      </c>
+      <c r="C43" s="1" t="str">
+        <v>Repairs &amp; Maintenance</v>
+      </c>
+      <c r="F43" s="1" t="str">
+        <v>+918805719505</v>
+      </c>
+      <c r="H43" s="1" t="str">
+        <v>11/468, Kapad Market Road, near Hotel Bellpepper, Vikas Nagar, Ichalkaranji</v>
+      </c>
+      <c r="I43" s="1" t="str">
+        <v>Computer, laptop and printer repairs; networking, CCTV and software setup enquiries</v>
+      </c>
+      <c r="J43" s="1" t="str">
+        <v>laptop repair, printer repair, CCTV installation, computer service, संगणक दुरुस्ती</v>
+      </c>
+      <c r="K43" s="1" t="str">
+        <v>https://www.manishainfo.in/terms</v>
+      </c>
+      <c r="L43" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M43" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N43" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="str">
+        <v>Shreecom Enterprises</v>
+      </c>
+      <c r="B44" s="1" t="str">
+        <v>Computer Sales &amp; Service</v>
+      </c>
+      <c r="C44" s="1" t="str">
+        <v>Repairs &amp; Maintenance</v>
+      </c>
+      <c r="F44" s="1" t="str">
+        <v>+919325811104</v>
+      </c>
+      <c r="H44" s="1" t="str">
+        <v>G-1, Girnar Apartment, Dhanya Lane, near Federal Bank, Ichalkaranji</v>
+      </c>
+      <c r="I44" s="1" t="str">
+        <v>Computer hardware and software support, custom desktop builds and data-recovery enquiries</v>
+      </c>
+      <c r="K44" s="1" t="str">
+        <v>https://www.shreecomenterprises.com/</v>
+      </c>
+      <c r="L44" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M44" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N44" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="str">
+        <v>FIE — Service Support</v>
+      </c>
+      <c r="B45" s="1" t="str">
+        <v>Testing Machine Service</v>
+      </c>
+      <c r="C45" s="1" t="str">
+        <v>Business &amp; Technical Services</v>
+      </c>
+      <c r="F45" s="1" t="str">
+        <v>+919850065630</v>
+      </c>
+      <c r="H45" s="1" t="str">
+        <v>Old Industrial Estate, Ichalkaranji; Yadrav facility</v>
+      </c>
+      <c r="I45" s="1" t="str">
+        <v>Testing-machine calibration, maintenance, repairs, spares and technical support</v>
+      </c>
+      <c r="K45" s="1" t="str">
+        <v>https://www.fietest.com/services.html</v>
+      </c>
+      <c r="L45" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M45" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N45" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="str">
+        <v>Yantra Pneumatics &amp; Equipments</v>
+      </c>
+      <c r="B46" s="1" t="str">
+        <v>Compressed Air Service</v>
+      </c>
+      <c r="C46" s="1" t="str">
+        <v>Business &amp; Technical Services</v>
+      </c>
+      <c r="F46" s="1" t="str">
+        <v>+919449850296</v>
+      </c>
+      <c r="G46" s="1" t="str">
+        <v>Published company contact; ask for the Ichalkaranji branch.</v>
+      </c>
+      <c r="H46" s="1" t="str">
+        <v>Ichalkaranji branch: 21/778, Jawahar Nagar, Decan Mill; Kolhapur head office</v>
+      </c>
+      <c r="I46" s="1" t="str">
+        <v>Compressor servicing, spares, compressed-air piping, leak testing and air audits</v>
+      </c>
+      <c r="K46" s="1" t="str">
+        <v>https://www.yantrapneumatics.com/</v>
+      </c>
+      <c r="L46" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M46" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N46" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="str">
+        <v>Navkar Fabtech</v>
+      </c>
+      <c r="B47" s="1" t="str">
+        <v>Weaving Equipment Service</v>
+      </c>
+      <c r="C47" s="1" t="str">
+        <v>Business &amp; Technical Services</v>
+      </c>
+      <c r="F47" s="1" t="str">
+        <v>+917448028501</v>
+      </c>
+      <c r="H47" s="1" t="str">
+        <v>Plot No. 270, Khanjire Industry, near VRL Godown, Industrial Estate, Ichalkaranji</v>
+      </c>
+      <c r="I47" s="1" t="str">
+        <v>Weaving accessories, technical support, spare parts and ultrasonic reed-cleaning enquiries</v>
+      </c>
+      <c r="K47" s="1" t="str">
+        <v>https://navkarfabtech.com/contact-us/</v>
+      </c>
+      <c r="L47" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M47" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N47" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="str">
+        <v>Develovation Enterprises</v>
+      </c>
+      <c r="B48" s="1" t="str">
+        <v>Civil Contractor</v>
+      </c>
+      <c r="C48" s="1" t="str">
+        <v>Home Interiors</v>
+      </c>
+      <c r="F48" s="1" t="str">
+        <v>+918884430303</v>
+      </c>
+      <c r="H48" s="1" t="str">
+        <v>7/266, Saraswati Market, Ichalkaranji</v>
+      </c>
+      <c r="I48" s="1" t="str">
+        <v>Civil contracting, RCC, foundations, renovation and industrial maintenance enquiries</v>
+      </c>
+      <c r="K48" s="1" t="str">
+        <v>https://develovation.org/</v>
+      </c>
+      <c r="L48" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M48" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N48" s="1" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="str">
+        <v>Ocean Computers</v>
+      </c>
+      <c r="B49" s="1" t="str">
+        <v>Computer &amp; CCTV Repair</v>
+      </c>
+      <c r="C49" s="1" t="str">
+        <v>Repairs &amp; Maintenance</v>
+      </c>
+      <c r="F49" s="1" t="str">
+        <v>+919067911777</v>
+      </c>
+      <c r="H49" s="1" t="str">
+        <v>19/84, Kolhapur Road, near ASC College, Ichalkaranji</v>
+      </c>
+      <c r="I49" s="1" t="str">
+        <v>Computer and laptop repair, printer repair and cartridge refilling, CCTV installation and maintenance</v>
+      </c>
+      <c r="K49" s="1" t="str">
+        <v>https://oceancomputerinstitute.in/sales-service</v>
+      </c>
+      <c r="L49" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M49" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N49" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="str">
+        <v>Tumbledry — Ichalkaranji Booking</v>
+      </c>
+      <c r="B50" s="1" t="str">
+        <v>Laundry &amp; Dry Cleaning</v>
+      </c>
+      <c r="C50" s="1" t="str">
+        <v>Home Help</v>
+      </c>
+      <c r="F50" s="1" t="str">
+        <v>+917677250250</v>
+      </c>
+      <c r="G50" s="1" t="str">
+        <v>Brand booking number published for Ichalkaranji; confirm pickup coverage and the local store before booking.</v>
+      </c>
+      <c r="H50" s="1" t="str">
+        <v>Kagwade Mala store, Sangli Naka–Shahpur Road, near Star Local Mart, Ichalkaranji</v>
+      </c>
+      <c r="I50" s="1" t="str">
+        <v>Laundry, dry cleaning, curtain, shoe and carpet-cleaning booking enquiries</v>
+      </c>
+      <c r="K50" s="1" t="str">
+        <v>https://tumbledry.in/best-dry-clean-shop-in-ichalkaranji/</v>
+      </c>
+      <c r="L50" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M50" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N50" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="str">
+        <v>Swapnshilp Consultants</v>
+      </c>
+      <c r="B51" s="1" t="str">
+        <v>Construction &amp; Design</v>
+      </c>
+      <c r="C51" s="1" t="str">
+        <v>Home Interiors</v>
+      </c>
+      <c r="F51" s="1" t="str">
+        <v>+919325830592</v>
+      </c>
+      <c r="H51" s="1" t="str">
+        <v>Ichalkaranji projects; Hulgeshwary Road / Station Road area</v>
+      </c>
+      <c r="I51" s="1" t="str">
+        <v>Building, construction-project and design enquiries</v>
+      </c>
+      <c r="K51" s="1" t="str">
+        <v>https://swapnashilpconsultants.com/project-details.php?id=7</v>
+      </c>
+      <c r="L51" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M51" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N51" s="1" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="str">
+        <v>Regal Paints</v>
+      </c>
+      <c r="B52" s="1" t="str">
+        <v>Paint Supplies</v>
+      </c>
+      <c r="C52" s="1" t="str">
+        <v>Home Improvement Supplies</v>
+      </c>
+      <c r="F52" s="1" t="str">
+        <v>+919822023699</v>
+      </c>
+      <c r="G52" s="1" t="str">
+        <v>Listed in the manufacturer's published 2024 dealer directory; confirm current contact details.</v>
+      </c>
+      <c r="H52" s="1" t="str">
+        <v>Near Peoples Bank, Bangala Road, Ichalkaranji</v>
+      </c>
+      <c r="I52" s="1" t="str">
+        <v>Paint dealer and home-painting material enquiries</v>
+      </c>
+      <c r="K52" s="1" t="str">
+        <v>https://nipponpaint.co.in/wp-content/uploads/2024/11/Maharashtra.pdf</v>
+      </c>
+      <c r="L52" s="1" t="str">
+        <v>Manufacturer dealer directory</v>
+      </c>
+      <c r="M52" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N52" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="str">
+        <v>Designers’ Group</v>
+      </c>
+      <c r="B53" s="1" t="str">
+        <v>Architect &amp; Interior Designer</v>
+      </c>
+      <c r="C53" s="1" t="str">
+        <v>Home Interiors</v>
+      </c>
+      <c r="F53" s="1" t="str">
+        <v>+912302434471</v>
+      </c>
+      <c r="H53" s="1" t="str">
+        <v>6/838, Khanjire Mala, Ichalkaranji</v>
+      </c>
+      <c r="I53" s="1" t="str">
+        <v>Architecture, building planning, interior and landscape-design enquiries</v>
+      </c>
+      <c r="K53" s="1" t="str">
+        <v>https://designersgrp.com/index.php</v>
+      </c>
+      <c r="L53" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M53" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N53" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="str">
+        <v>Sreem Industries</v>
+      </c>
+      <c r="B54" s="1" t="str">
+        <v>Shop Furniture Fabrication</v>
+      </c>
+      <c r="C54" s="1" t="str">
+        <v>Business &amp; Technical Services</v>
+      </c>
+      <c r="F54" s="1" t="str">
+        <v>+919561383144</v>
+      </c>
+      <c r="H54" s="1" t="str">
+        <v>Ichalkaranji and surrounding area</v>
+      </c>
+      <c r="I54" s="1" t="str">
+        <v>Made-to-order furniture and storage for medical stores, grocery shops and clothing shops</v>
+      </c>
+      <c r="K54" s="1" t="str">
+        <v>https://sreem-industries.ueniweb.com/</v>
+      </c>
+      <c r="L54" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M54" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N54" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="str">
+        <v>Bombay Andhra Transport — Ichalkaranji</v>
+      </c>
+      <c r="B55" s="1" t="str">
+        <v>Goods Transport</v>
+      </c>
+      <c r="C55" s="1" t="str">
+        <v>Transport &amp; Travel</v>
+      </c>
+      <c r="F55" s="1" t="str">
+        <v>+917020254150</v>
+      </c>
+      <c r="H55" s="1" t="str">
+        <v>Ward No. 23, Plot No. 403, Khanjire Industrial Estate, near Sana Engineering, Ichalkaranji</v>
+      </c>
+      <c r="I55" s="1" t="str">
+        <v>Goods transport and freight-booking enquiries</v>
+      </c>
+      <c r="K55" s="1" t="str">
+        <v>https://batps.com/citys.php?sid=1</v>
+      </c>
+      <c r="L55" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M55" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N55" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="str">
+        <v>BIS — Kolhapur Area Security</v>
+      </c>
+      <c r="B56" s="1" t="str">
+        <v>Security Guard Services</v>
+      </c>
+      <c r="C56" s="1" t="str">
+        <v>Building Services</v>
+      </c>
+      <c r="F56" s="1" t="str">
+        <v>+919322875680</v>
+      </c>
+      <c r="H56" s="1" t="str">
+        <v>Kolhapur office advertising service coverage in Ichalkaranji</v>
+      </c>
+      <c r="I56" s="1" t="str">
+        <v>Security-guard and site-security service enquiries for commercial, industrial and residential sites</v>
+      </c>
+      <c r="K56" s="1" t="str">
+        <v>https://www.bombayintegrated.com/security-services-kolhapur</v>
+      </c>
+      <c r="L56" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M56" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N56" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="str">
+        <v>Shri Hospital Equipment</v>
+      </c>
+      <c r="B57" s="1" t="str">
+        <v>Hospital Furniture &amp; Equipment</v>
+      </c>
+      <c r="C57" s="1" t="str">
+        <v>Healthcare</v>
+      </c>
+      <c r="F57" s="1" t="str">
+        <v>+918380001702</v>
+      </c>
+      <c r="H57" s="1" t="str">
+        <v>Siddeshwar Colony, Shahapur, 23/112 Jawahar Nagar, Industrial Estate, Ichalkaranji</v>
+      </c>
+      <c r="I57" s="1" t="str">
+        <v>Hospital furniture and equipment supply enquiries</v>
+      </c>
+      <c r="K57" s="1" t="str">
+        <v>https://shriequipment.com/contact-us/</v>
+      </c>
+      <c r="L57" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M57" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N57" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="str">
+        <v>PALM Diagnostics &amp; Heart Care Clinic</v>
+      </c>
+      <c r="B58" s="1" t="str">
+        <v>Diagnostic &amp; Clinic Enquiries</v>
+      </c>
+      <c r="C58" s="1" t="str">
+        <v>Healthcare</v>
+      </c>
+      <c r="F58" s="1" t="str">
+        <v>+912302429898</v>
+      </c>
+      <c r="H58" s="1" t="str">
+        <v>Ichalkaranji</v>
+      </c>
+      <c r="I58" s="1" t="str">
+        <v>Diagnostic centre and clinic appointment enquiries</v>
+      </c>
+      <c r="K58" s="1" t="str">
+        <v>https://palmdiagnosticsheartcareclinic.com/</v>
+      </c>
+      <c r="L58" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M58" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N58" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="str">
+        <v>Manchester Hospital</v>
+      </c>
+      <c r="B59" s="1" t="str">
+        <v>Hospital Enquiries</v>
+      </c>
+      <c r="C59" s="1" t="str">
+        <v>Healthcare</v>
+      </c>
+      <c r="F59" s="1" t="str">
+        <v>+919823371255</v>
+      </c>
+      <c r="H59" s="1" t="str">
+        <v>Behind Yadrav petrol pump, Yadrav Phata, Ichalkaranji</v>
+      </c>
+      <c r="I59" s="1" t="str">
+        <v>Hospital appointment and facility enquiries</v>
+      </c>
+      <c r="K59" s="1" t="str">
+        <v>https://manchestermsp.wixsite.com/manchesterhospital</v>
+      </c>
+      <c r="L59" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M59" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N59" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="str">
+        <v>Bhatkanti Tours — Ichalkaranji</v>
+      </c>
+      <c r="B60" s="1" t="str">
+        <v>Travel Agency</v>
+      </c>
+      <c r="C60" s="1" t="str">
+        <v>Transport &amp; Travel</v>
+      </c>
+      <c r="F60" s="1" t="str">
+        <v>+919420492515</v>
+      </c>
+      <c r="H60" s="1" t="str">
+        <v>12/59, Gala No. 9, Kalpana Talkies Building, Bangla Road, Ichalkaranji</v>
+      </c>
+      <c r="I60" s="1" t="str">
+        <v>Tour bookings, travel planning and holiday enquiries</v>
+      </c>
+      <c r="K60" s="1" t="str">
+        <v>https://bhatkantitours.in/contact-us/</v>
+      </c>
+      <c r="L60" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M60" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N60" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="str">
+        <v>Bellpepper Catering Services</v>
+      </c>
+      <c r="B61" s="1" t="str">
+        <v>Caterer</v>
+      </c>
+      <c r="C61" s="1" t="str">
+        <v>Events &amp; Catering</v>
+      </c>
+      <c r="F61" s="1" t="str">
+        <v>+919860440366</v>
+      </c>
+      <c r="H61" s="1" t="str">
+        <v>Chogule Building, opposite Kapad Market, Ichalkaranji</v>
+      </c>
+      <c r="I61" s="1" t="str">
+        <v>Vegetarian catering enquiries for weddings, birthdays, house parties and corporate events</v>
+      </c>
+      <c r="K61" s="1" t="str">
+        <v>https://bellpeppercatering.com/</v>
+      </c>
+      <c r="L61" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M61" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N61" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="str">
+        <v>Magdum Eye &amp; Dental Hospital</v>
+      </c>
+      <c r="B62" s="1" t="str">
+        <v>Eye &amp; Dental Appointments</v>
+      </c>
+      <c r="C62" s="1" t="str">
+        <v>Healthcare</v>
+      </c>
+      <c r="F62" s="1" t="str">
+        <v>+912302424466</v>
+      </c>
+      <c r="H62" s="1" t="str">
+        <v>Fire Fighter Road, Ichalkaranji</v>
+      </c>
+      <c r="I62" s="1" t="str">
+        <v>Eye and dental hospital appointment enquiries</v>
+      </c>
+      <c r="K62" s="1" t="str">
+        <v>https://www.magdumhospital.com/contact-us.php</v>
+      </c>
+      <c r="L62" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M62" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N62" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="str">
+        <v>Gobo Tours — Heena Tours Franchise</v>
+      </c>
+      <c r="B63" s="1" t="str">
+        <v>Travel Agency</v>
+      </c>
+      <c r="C63" s="1" t="str">
+        <v>Transport &amp; Travel</v>
+      </c>
+      <c r="F63" s="1" t="str">
+        <v>+912302425294</v>
+      </c>
+      <c r="H63" s="1" t="str">
+        <v>8/218, Kapad Market, Ichalkaranji</v>
+      </c>
+      <c r="I63" s="1" t="str">
+        <v>Tour and holiday booking enquiries</v>
+      </c>
+      <c r="K63" s="1" t="str">
+        <v>https://www.heenatours.in/branches</v>
+      </c>
+      <c r="L63" s="1" t="str">
+        <v>Brand branch directory</v>
+      </c>
+      <c r="M63" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N63" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="str">
+        <v>Mauli Caterers</v>
+      </c>
+      <c r="B64" s="1" t="str">
+        <v>Caterer</v>
+      </c>
+      <c r="C64" s="1" t="str">
+        <v>Events &amp; Catering</v>
+      </c>
+      <c r="F64" s="1" t="str">
+        <v>+919890036604</v>
+      </c>
+      <c r="H64" s="1" t="str">
+        <v>Ichalkaranji, Maharashtra 416115</v>
+      </c>
+      <c r="I64" s="1" t="str">
+        <v>Catering enquiries for local functions</v>
+      </c>
+      <c r="K64" s="1" t="str">
+        <v>https://mauli-caterers.ueniweb.com/services/range-of-services/catering-26490428</v>
+      </c>
+      <c r="L64" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M64" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N64" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="str">
+        <v>Sunvolt Enterprises</v>
+      </c>
+      <c r="B65" s="1" t="str">
+        <v>Solar Installation</v>
+      </c>
+      <c r="C65" s="1" t="str">
+        <v>Solar &amp; Energy</v>
+      </c>
+      <c r="F65" s="1" t="str">
+        <v>+919225819909</v>
+      </c>
+      <c r="H65" s="1" t="str">
+        <v>Jaysingpur-based provider listing completed work in Ichalkaranji</v>
+      </c>
+      <c r="I65" s="1" t="str">
+        <v>Residential and commercial solar installation and solar-equipment enquiries</v>
+      </c>
+      <c r="K65" s="1" t="str">
+        <v>https://sunvoltenterprises.com/</v>
+      </c>
+      <c r="L65" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M65" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N65" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="str">
+        <v>Madhavbaug — Ichalkaranji Clinic</v>
+      </c>
+      <c r="B66" s="1" t="str">
+        <v>Clinic Appointments</v>
+      </c>
+      <c r="C66" s="1" t="str">
+        <v>Healthcare</v>
+      </c>
+      <c r="F66" s="1" t="str">
+        <v>+919850080092</v>
+      </c>
+      <c r="H66" s="1" t="str">
+        <v>Malkar Building, opposite Weekly Market, near Uttam Prakash Talkies, Ichalkaranji</v>
+      </c>
+      <c r="I66" s="1" t="str">
+        <v>Clinic appointment and consultation enquiries</v>
+      </c>
+      <c r="K66" s="1" t="str">
+        <v>https://madhavbaug.org/clinic/ichalkaranji-kolhapur</v>
+      </c>
+      <c r="L66" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M66" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N66" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="str">
+        <v>Heritage Hall — DeepNanda Group</v>
+      </c>
+      <c r="B67" s="1" t="str">
+        <v>Event Venue</v>
+      </c>
+      <c r="C67" s="1" t="str">
+        <v>Events &amp; Catering</v>
+      </c>
+      <c r="F67" s="1" t="str">
+        <v>+919175166779</v>
+      </c>
+      <c r="H67" s="1" t="str">
+        <v>Gat No. 233, Ichalkaranji–Shiradwad Road, Shiradwad, near Ichalkaranji</v>
+      </c>
+      <c r="I67" s="1" t="str">
+        <v>Wedding, function, conference and venue-booking enquiries</v>
+      </c>
+      <c r="K67" s="1" t="str">
+        <v>https://deepnandagroup.com/heritage_hall.php</v>
+      </c>
+      <c r="L67" s="1" t="str">
+        <v>Business website</v>
+      </c>
+      <c r="M67" s="1" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="N67" s="1" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N67"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>